<commit_message>
Deploy expandable Vistavki detail downloads
</commit_message>
<xml_diff>
--- a/data/processed/expomap_portal/exports/expomap_moscow_expo_2026_public_events.xlsx
+++ b/data/processed/expomap_portal/exports/expomap_moscow_expo_2026_public_events.xlsx
@@ -18282,8 +18282,16 @@
           <t>https://expomap.ru/expo/logistika-expo/</t>
         </is>
       </c>
-      <c r="Q187" t="inlineStr"/>
-      <c r="R187" t="inlineStr"/>
+      <c r="Q187" t="inlineStr">
+        <is>
+          <t>https://logistika-expo.ru/</t>
+        </is>
+      </c>
+      <c r="R187" t="inlineStr">
+        <is>
+          <t>https://logistika-expo.ru/</t>
+        </is>
+      </c>
       <c r="S187" t="inlineStr">
         <is>
           <t>no</t>

</xml_diff>

<commit_message>
Deploy EcoGorod ZOZH portal update
</commit_message>
<xml_diff>
--- a/data/processed/expomap_portal/exports/expomap_moscow_expo_2026_public_events.xlsx
+++ b/data/processed/expomap_portal/exports/expomap_moscow_expo_2026_public_events.xlsx
@@ -3185,12 +3185,12 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>http://измайловошуз.рф</t>
+          <t>https://izmailovoshoes.ru/en/</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>http://измайловошуз.рф</t>
+          <t>https://izmailovoshoes.ru/en/</t>
         </is>
       </c>
       <c r="X24" t="inlineStr">
@@ -8245,8 +8245,16 @@
           <t>https://expomap.ru/expo/moscow-overseas-property-investment-show/</t>
         </is>
       </c>
-      <c r="V67" t="inlineStr"/>
-      <c r="W67" t="inlineStr"/>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>https://investshow.ru/eng/</t>
+        </is>
+      </c>
+      <c r="W67" t="inlineStr">
+        <is>
+          <t>https://investshow.ru/eng/</t>
+        </is>
+      </c>
       <c r="X67" t="inlineStr">
         <is>
           <t>no</t>
@@ -12122,12 +12130,12 @@
       </c>
       <c r="V101" t="inlineStr">
         <is>
-          <t>https://wedding-fashion.ru/</t>
+          <t>https://wfmexpo.ru/</t>
         </is>
       </c>
       <c r="W101" t="inlineStr">
         <is>
-          <t>https://wedding-fashion.ru/</t>
+          <t>https://wfmexpo.ru/</t>
         </is>
       </c>
       <c r="X101" t="inlineStr">
@@ -21652,8 +21660,16 @@
           <t>https://expomap.ru/expo/metallokonstruktsii/</t>
         </is>
       </c>
-      <c r="V183" t="inlineStr"/>
-      <c r="W183" t="inlineStr"/>
+      <c r="V183" t="inlineStr">
+        <is>
+          <t>https://mc-expo.ru/en</t>
+        </is>
+      </c>
+      <c r="W183" t="inlineStr">
+        <is>
+          <t>https://mc-expo.ru/en</t>
+        </is>
+      </c>
       <c r="X183" t="inlineStr">
         <is>
           <t>no</t>
@@ -21887,8 +21903,16 @@
           <t>https://expomap.ru/expo/ctt-expo/</t>
         </is>
       </c>
-      <c r="V185" t="inlineStr"/>
-      <c r="W185" t="inlineStr"/>
+      <c r="V185" t="inlineStr">
+        <is>
+          <t>https://ctt-expo.ru/about-eng</t>
+        </is>
+      </c>
+      <c r="W185" t="inlineStr">
+        <is>
+          <t>https://ctt-expo.ru/about-eng</t>
+        </is>
+      </c>
       <c r="X185" t="inlineStr">
         <is>
           <t>no</t>
@@ -34199,8 +34223,16 @@
           <t>https://expomap.ru/expo/jarmarka-uk/</t>
         </is>
       </c>
-      <c r="V288" t="inlineStr"/>
-      <c r="W288" t="inlineStr"/>
+      <c r="V288" t="inlineStr">
+        <is>
+          <t>https://okron.ru/exhibition/2026</t>
+        </is>
+      </c>
+      <c r="W288" t="inlineStr">
+        <is>
+          <t>https://okron.ru/exhibition/2026</t>
+        </is>
+      </c>
       <c r="X288" t="inlineStr">
         <is>
           <t>no</t>
@@ -38614,12 +38646,12 @@
       </c>
       <c r="V325" t="inlineStr">
         <is>
-          <t>https://vezdehoder.ru/?ysclid=mimwdpol3t901117147</t>
+          <t>https://vezdehoder.ru/</t>
         </is>
       </c>
       <c r="W325" t="inlineStr">
         <is>
-          <t>https://vezdehoder.ru/?ysclid=mimwdpol3t901117147</t>
+          <t>https://vezdehoder.ru/</t>
         </is>
       </c>
       <c r="X325" t="inlineStr">

</xml_diff>

<commit_message>
Deploy SobMaExpo Global Ingredients portal data
</commit_message>
<xml_diff>
--- a/data/processed/expomap_portal/exports/expomap_moscow_expo_2026_public_events.xlsx
+++ b/data/processed/expomap_portal/exports/expomap_moscow_expo_2026_public_events.xlsx
@@ -1004,16 +1004,8 @@
           <t>https://expomap.ru/expo/sport-casual-moscow/</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>https://sportcasualmoscow.ru/?utm_source=expomap</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>https://sportcasualmoscow.ru/?utm_source=expomap</t>
-        </is>
-      </c>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
       <c r="X5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2039,16 +2031,8 @@
           <t>https://expomap.ru/expo/additive-minded/</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>https://ruplastica.ru/news/20250916-additive-minded-2026-vystavka-gde-promyshlennost-vstrechaetsya-s-3d-pechatyu</t>
-        </is>
-      </c>
-      <c r="W14" t="inlineStr">
-        <is>
-          <t>https://ruplastica.ru/news/20250916-additive-minded-2026-vystavka-gde-promyshlennost-vstrechaetsya-s-3d-pechatyu</t>
-        </is>
-      </c>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr"/>
       <c r="X14" t="inlineStr">
         <is>
           <t>no</t>
@@ -3018,12 +3002,12 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>{"beverage_exclusion": ["Вино", "Кофе", "Напитки", "Чай"], "broad": ["Пищевая индустрия", "Сельское хозяйство"], "negative": [], "official_url": ["Продэкспо"], "positive": ["Деликатесы", "Детское питание", "Кондитерские изделия", "Корма", "Молочная индустрия", "Мороженое", "Овощи", "Пищевые добавки", "Пищевые ингредиенты", "Продэкспо", "Рыба", "Упаковка", "Фрукты", "Фрукты и овощи"]}</t>
+          <t>{"beverage_exclusion": ["Вино", "Кофе", "Напитки", "Чай"], "broad": ["Пищевая индустрия", "Сельское хозяйство"], "negative": [], "official_url": [], "positive": ["Деликатесы", "Детское питание", "Кондитерские изделия", "Корма", "Молочная индустрия", "Мороженое", "Овощи", "Пищевые добавки", "Пищевые ингредиенты", "Рыба", "Упаковка", "Фрукты", "Фрукты и овощи"]}</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>consumer_goods_retail; food_agri_products_non_beverage; official_url_positive_cue; packaging_printing_label_marking</t>
+          <t>consumer_goods_retail; food_agri_products_non_beverage; packaging_printing_label_marking</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -3073,16 +3057,8 @@
           <t>https://expomap.ru/expo/prodexpo/2026/</t>
         </is>
       </c>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>https://www.prod-expo.ru/</t>
-        </is>
-      </c>
-      <c r="W23" t="inlineStr">
-        <is>
-          <t>https://www.prod-expo.ru/</t>
-        </is>
-      </c>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="inlineStr"/>
       <c r="X23" t="inlineStr">
         <is>
           <t>no</t>
@@ -3183,16 +3159,8 @@
           <t>https://expomap.ru/expo/izmajlovo-shuz/</t>
         </is>
       </c>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>https://izmailovoshoes.ru/en/</t>
-        </is>
-      </c>
-      <c r="W24" t="inlineStr">
-        <is>
-          <t>https://izmailovoshoes.ru/en/</t>
-        </is>
-      </c>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr"/>
       <c r="X24" t="inlineStr">
         <is>
           <t>no</t>
@@ -4119,16 +4087,8 @@
           <t>https://expomap.ru/expo/cstbpromedia/</t>
         </is>
       </c>
-      <c r="V32" t="inlineStr">
-        <is>
-          <t>https://cstb.ru/</t>
-        </is>
-      </c>
-      <c r="W32" t="inlineStr">
-        <is>
-          <t>https://cstb.ru/</t>
-        </is>
-      </c>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr"/>
       <c r="X32" t="inlineStr">
         <is>
           <t>no</t>
@@ -4245,16 +4205,8 @@
           <t>https://expomap.ru/expo/cpm-collection-premiere-moscow/2026/feb/</t>
         </is>
       </c>
-      <c r="V33" t="inlineStr">
-        <is>
-          <t>https://cpm-moscow.com/?lang=ru/?erid=2VfnxyWEqvi</t>
-        </is>
-      </c>
-      <c r="W33" t="inlineStr">
-        <is>
-          <t>https://cpm-moscow.com/?lang=ru/?erid=2VfnxyWEqvi</t>
-        </is>
-      </c>
+      <c r="V33" t="inlineStr"/>
+      <c r="W33" t="inlineStr"/>
       <c r="X33" t="inlineStr">
         <is>
           <t>no</t>
@@ -4374,16 +4326,8 @@
           <t>https://expomap.ru/expo/miof/</t>
         </is>
       </c>
-      <c r="V34" t="inlineStr">
-        <is>
-          <t>http://www.optica-expo.ru/optica/exhibition/</t>
-        </is>
-      </c>
-      <c r="W34" t="inlineStr">
-        <is>
-          <t>http://www.optica-expo.ru/optica/exhibition/</t>
-        </is>
-      </c>
+      <c r="V34" t="inlineStr"/>
+      <c r="W34" t="inlineStr"/>
       <c r="X34" t="inlineStr">
         <is>
           <t>no</t>
@@ -4812,16 +4756,8 @@
           <t>https://expomap.ru/expo/graduate-awards/</t>
         </is>
       </c>
-      <c r="V38" t="inlineStr">
-        <is>
-          <t>https://clck.ru/3Meg3N</t>
-        </is>
-      </c>
-      <c r="W38" t="inlineStr">
-        <is>
-          <t>https://clck.ru/3Meg3N</t>
-        </is>
-      </c>
+      <c r="V38" t="inlineStr"/>
+      <c r="W38" t="inlineStr"/>
       <c r="X38" t="inlineStr">
         <is>
           <t>no</t>
@@ -4943,16 +4879,8 @@
           <t>https://expomap.ru/expo/ohota-i-rybolovstvo-na-rusi/</t>
         </is>
       </c>
-      <c r="V39" t="inlineStr">
-        <is>
-          <t>https://www.hunting-expo.ru/</t>
-        </is>
-      </c>
-      <c r="W39" t="inlineStr">
-        <is>
-          <t>https://www.hunting-expo.ru/</t>
-        </is>
-      </c>
+      <c r="V39" t="inlineStr"/>
+      <c r="W39" t="inlineStr"/>
       <c r="X39" t="inlineStr">
         <is>
           <t>no</t>
@@ -5645,16 +5573,8 @@
           <t>https://expomap.ru/expo/mir-ohoty-i-rybalki/</t>
         </is>
       </c>
-      <c r="V45" t="inlineStr">
-        <is>
-          <t>https://www.huntfishexpo.ru/</t>
-        </is>
-      </c>
-      <c r="W45" t="inlineStr">
-        <is>
-          <t>https://www.huntfishexpo.ru/</t>
-        </is>
-      </c>
+      <c r="V45" t="inlineStr"/>
+      <c r="W45" t="inlineStr"/>
       <c r="X45" t="inlineStr">
         <is>
           <t>no</t>
@@ -5756,16 +5676,8 @@
           <t>https://expomap.ru/expo/bizhufest/</t>
         </is>
       </c>
-      <c r="V46" t="inlineStr">
-        <is>
-          <t>https://bijou-moscow.com/</t>
-        </is>
-      </c>
-      <c r="W46" t="inlineStr">
-        <is>
-          <t>https://bijou-moscow.com/</t>
-        </is>
-      </c>
+      <c r="V46" t="inlineStr"/>
+      <c r="W46" t="inlineStr"/>
       <c r="X46" t="inlineStr">
         <is>
           <t>no</t>
@@ -5989,16 +5901,8 @@
           <t>https://expomap.ru/expo/zhit-krasivo/</t>
         </is>
       </c>
-      <c r="V48" t="inlineStr">
-        <is>
-          <t>https://zkrasivo.ru/</t>
-        </is>
-      </c>
-      <c r="W48" t="inlineStr">
-        <is>
-          <t>https://zkrasivo.ru/</t>
-        </is>
-      </c>
+      <c r="V48" t="inlineStr"/>
+      <c r="W48" t="inlineStr"/>
       <c r="X48" t="inlineStr">
         <is>
           <t>no</t>
@@ -6210,16 +6114,8 @@
           <t>https://expomap.ru/expo/festival-stoljarnogo-dela/</t>
         </is>
       </c>
-      <c r="V50" t="inlineStr">
-        <is>
-          <t>https://rubankov.ru/festival/</t>
-        </is>
-      </c>
-      <c r="W50" t="inlineStr">
-        <is>
-          <t>https://rubankov.ru/festival/</t>
-        </is>
-      </c>
+      <c r="V50" t="inlineStr"/>
+      <c r="W50" t="inlineStr"/>
       <c r="X50" t="inlineStr">
         <is>
           <t>no</t>
@@ -6324,16 +6220,8 @@
           <t>https://expomap.ru/expo/mybabyko/</t>
         </is>
       </c>
-      <c r="V51" t="inlineStr">
-        <is>
-          <t>https://mybabyko.ru/</t>
-        </is>
-      </c>
-      <c r="W51" t="inlineStr">
-        <is>
-          <t>https://mybabyko.ru/</t>
-        </is>
-      </c>
+      <c r="V51" t="inlineStr"/>
+      <c r="W51" t="inlineStr"/>
       <c r="X51" t="inlineStr">
         <is>
           <t>no</t>
@@ -6445,16 +6333,8 @@
           <t>https://expomap.ru/expo/sobytie-goda/</t>
         </is>
       </c>
-      <c r="V52" t="inlineStr">
-        <is>
-          <t>https://eventawardsrussia.com/?utm_source=expomap</t>
-        </is>
-      </c>
-      <c r="W52" t="inlineStr">
-        <is>
-          <t>https://eventawardsrussia.com/?utm_source=expomap</t>
-        </is>
-      </c>
+      <c r="V52" t="inlineStr"/>
+      <c r="W52" t="inlineStr"/>
       <c r="X52" t="inlineStr">
         <is>
           <t>no</t>
@@ -6829,16 +6709,8 @@
           <t>https://expomap.ru/expo/tekstillegprom/2026/mar/</t>
         </is>
       </c>
-      <c r="V55" t="inlineStr">
-        <is>
-          <t>https://textilexpo.ru/</t>
-        </is>
-      </c>
-      <c r="W55" t="inlineStr">
-        <is>
-          <t>https://textilexpo.ru/</t>
-        </is>
-      </c>
+      <c r="V55" t="inlineStr"/>
+      <c r="W55" t="inlineStr"/>
       <c r="X55" t="inlineStr">
         <is>
           <t>no</t>
@@ -6955,16 +6827,8 @@
           <t>https://expomap.ru/expo/textile-collection-moscow/</t>
         </is>
       </c>
-      <c r="V56" t="inlineStr">
-        <is>
-          <t>https://textile-collection.com/?utm_medium=partner_free&amp;utm_campaign=expomap</t>
-        </is>
-      </c>
-      <c r="W56" t="inlineStr">
-        <is>
-          <t>https://textile-collection.com/?utm_medium=partner_free&amp;utm_campaign=expomap</t>
-        </is>
-      </c>
+      <c r="V56" t="inlineStr"/>
+      <c r="W56" t="inlineStr"/>
       <c r="X56" t="inlineStr">
         <is>
           <t>no</t>
@@ -7781,16 +7645,8 @@
           <t>https://expomap.ru/expo/navigatsija-i-svjaz-v-osobyh-uslovijah/</t>
         </is>
       </c>
-      <c r="V63" t="inlineStr">
-        <is>
-          <t>https://navicomexpo.ru/</t>
-        </is>
-      </c>
-      <c r="W63" t="inlineStr">
-        <is>
-          <t>https://navicomexpo.ru/</t>
-        </is>
-      </c>
+      <c r="V63" t="inlineStr"/>
+      <c r="W63" t="inlineStr"/>
       <c r="X63" t="inlineStr">
         <is>
           <t>no</t>
@@ -7900,16 +7756,8 @@
           <t>https://expomap.ru/expo/eco-beauty-expo/2026/mar/</t>
         </is>
       </c>
-      <c r="V64" t="inlineStr">
-        <is>
-          <t>https://eco-beauty-expo.ru/?utm_source=expomap</t>
-        </is>
-      </c>
-      <c r="W64" t="inlineStr">
-        <is>
-          <t>https://eco-beauty-expo.ru/?utm_source=expomap</t>
-        </is>
-      </c>
+      <c r="V64" t="inlineStr"/>
+      <c r="W64" t="inlineStr"/>
       <c r="X64" t="inlineStr">
         <is>
           <t>no</t>
@@ -8018,16 +7866,8 @@
           <t>https://expomap.ru/expo/best-russia/</t>
         </is>
       </c>
-      <c r="V65" t="inlineStr">
-        <is>
-          <t>https://www.bestrussia.org/ru</t>
-        </is>
-      </c>
-      <c r="W65" t="inlineStr">
-        <is>
-          <t>https://www.bestrussia.org/ru</t>
-        </is>
-      </c>
+      <c r="V65" t="inlineStr"/>
+      <c r="W65" t="inlineStr"/>
       <c r="X65" t="inlineStr">
         <is>
           <t>no</t>
@@ -8245,16 +8085,8 @@
           <t>https://expomap.ru/expo/moscow-overseas-property-investment-show/</t>
         </is>
       </c>
-      <c r="V67" t="inlineStr">
-        <is>
-          <t>https://investshow.ru/eng/</t>
-        </is>
-      </c>
-      <c r="W67" t="inlineStr">
-        <is>
-          <t>https://investshow.ru/eng/</t>
-        </is>
-      </c>
+      <c r="V67" t="inlineStr"/>
+      <c r="W67" t="inlineStr"/>
       <c r="X67" t="inlineStr">
         <is>
           <t>no</t>
@@ -8354,16 +8186,8 @@
           <t>https://expomap.ru/expo/pro-chastnoe-dlya-roditelej/2026/</t>
         </is>
       </c>
-      <c r="V68" t="inlineStr">
-        <is>
-          <t>https://xn--80akxccchkj1c.xn--p1ai/?ysclid=mm35qy0qmv243008381</t>
-        </is>
-      </c>
-      <c r="W68" t="inlineStr">
-        <is>
-          <t>https://xn--80akxccchkj1c.xn--p1ai/?ysclid=mm35qy0qmv243008381</t>
-        </is>
-      </c>
+      <c r="V68" t="inlineStr"/>
+      <c r="W68" t="inlineStr"/>
       <c r="X68" t="inlineStr">
         <is>
           <t>no</t>
@@ -9926,16 +9750,8 @@
           <t>https://expomap.ru/expo/design/2026/mar/</t>
         </is>
       </c>
-      <c r="V82" t="inlineStr">
-        <is>
-          <t>https://design-plus.ru/</t>
-        </is>
-      </c>
-      <c r="W82" t="inlineStr">
-        <is>
-          <t>https://design-plus.ru/</t>
-        </is>
-      </c>
+      <c r="V82" t="inlineStr"/>
+      <c r="W82" t="inlineStr"/>
       <c r="X82" t="inlineStr">
         <is>
           <t>no</t>
@@ -10391,16 +10207,8 @@
           <t>https://expomap.ru/expo/rappa-expo/2026/mar/</t>
         </is>
       </c>
-      <c r="V86" t="inlineStr">
-        <is>
-          <t>https://raapa-expo.ru/</t>
-        </is>
-      </c>
-      <c r="W86" t="inlineStr">
-        <is>
-          <t>https://raapa-expo.ru/</t>
-        </is>
-      </c>
+      <c r="V86" t="inlineStr"/>
+      <c r="W86" t="inlineStr"/>
       <c r="X86" t="inlineStr">
         <is>
           <t>no</t>
@@ -10514,16 +10322,8 @@
           <t>https://expomap.ru/expo/robototechnika-i-iskusstvennyj-intellekt/</t>
         </is>
       </c>
-      <c r="V87" t="inlineStr">
-        <is>
-          <t>https://raiexpo.ru/</t>
-        </is>
-      </c>
-      <c r="W87" t="inlineStr">
-        <is>
-          <t>https://raiexpo.ru/</t>
-        </is>
-      </c>
+      <c r="V87" t="inlineStr"/>
+      <c r="W87" t="inlineStr"/>
       <c r="X87" t="inlineStr">
         <is>
           <t>no</t>
@@ -10727,16 +10527,8 @@
           <t>https://expomap.ru/expo/lifestyle-expo/</t>
         </is>
       </c>
-      <c r="V89" t="inlineStr">
-        <is>
-          <t>https://school.smart-and-talented.ru/lifestyleexpo2026</t>
-        </is>
-      </c>
-      <c r="W89" t="inlineStr">
-        <is>
-          <t>https://school.smart-and-talented.ru/lifestyleexpo2026</t>
-        </is>
-      </c>
+      <c r="V89" t="inlineStr"/>
+      <c r="W89" t="inlineStr"/>
       <c r="X89" t="inlineStr">
         <is>
           <t>no</t>
@@ -10939,16 +10731,8 @@
           <t>https://expomap.ru/expo/otkrytyj-sklad/</t>
         </is>
       </c>
-      <c r="V91" t="inlineStr">
-        <is>
-          <t>https://openshowroom.ru/menswomens_and_childrens_clothingfootwear_and_accessories</t>
-        </is>
-      </c>
-      <c r="W91" t="inlineStr">
-        <is>
-          <t>https://openshowroom.ru/menswomens_and_childrens_clothingfootwear_and_accessories</t>
-        </is>
-      </c>
+      <c r="V91" t="inlineStr"/>
+      <c r="W91" t="inlineStr"/>
       <c r="X91" t="inlineStr">
         <is>
           <t>no</t>
@@ -11563,16 +11347,8 @@
           <t>https://expomap.ru/expo/profbeauty-expo/</t>
         </is>
       </c>
-      <c r="V96" t="inlineStr">
-        <is>
-          <t>https://profbeauty-expo.ru/?utm_source=expomap</t>
-        </is>
-      </c>
-      <c r="W96" t="inlineStr">
-        <is>
-          <t>https://profbeauty-expo.ru/?utm_source=expomap</t>
-        </is>
-      </c>
+      <c r="V96" t="inlineStr"/>
+      <c r="W96" t="inlineStr"/>
       <c r="X96" t="inlineStr">
         <is>
           <t>no</t>
@@ -11687,16 +11463,8 @@
           <t>https://expomap.ru/expo/rusartstil/</t>
         </is>
       </c>
-      <c r="V97" t="inlineStr">
-        <is>
-          <t>https://www.expo-resurs.ru</t>
-        </is>
-      </c>
-      <c r="W97" t="inlineStr">
-        <is>
-          <t>https://www.expo-resurs.ru</t>
-        </is>
-      </c>
+      <c r="V97" t="inlineStr"/>
+      <c r="W97" t="inlineStr"/>
       <c r="X97" t="inlineStr">
         <is>
           <t>no</t>
@@ -11903,16 +11671,8 @@
           <t>https://expomap.ru/expo/luchshij-otso-rossii-i-sng/</t>
         </is>
       </c>
-      <c r="V99" t="inlineStr">
-        <is>
-          <t>https://clck.ru/3FBhgV</t>
-        </is>
-      </c>
-      <c r="W99" t="inlineStr">
-        <is>
-          <t>https://clck.ru/3FBhgV</t>
-        </is>
-      </c>
+      <c r="V99" t="inlineStr"/>
+      <c r="W99" t="inlineStr"/>
       <c r="X99" t="inlineStr">
         <is>
           <t>no</t>
@@ -12128,16 +11888,8 @@
           <t>https://expomap.ru/expo/wedding-fashion-moscow/</t>
         </is>
       </c>
-      <c r="V101" t="inlineStr">
-        <is>
-          <t>https://wfmexpo.ru/</t>
-        </is>
-      </c>
-      <c r="W101" t="inlineStr">
-        <is>
-          <t>https://wfmexpo.ru/</t>
-        </is>
-      </c>
+      <c r="V101" t="inlineStr"/>
+      <c r="W101" t="inlineStr"/>
       <c r="X101" t="inlineStr">
         <is>
           <t>no</t>
@@ -12611,16 +12363,8 @@
           <t>https://expomap.ru/expo/ekspertnaya-gostinaya/</t>
         </is>
       </c>
-      <c r="V105" t="inlineStr">
-        <is>
-          <t>https://forumsmartcity.ru/mosbuild2026/?utm_source=expomap</t>
-        </is>
-      </c>
-      <c r="W105" t="inlineStr">
-        <is>
-          <t>https://forumsmartcity.ru/mosbuild2026/?utm_source=expomap</t>
-        </is>
-      </c>
+      <c r="V105" t="inlineStr"/>
+      <c r="W105" t="inlineStr"/>
       <c r="X105" t="inlineStr">
         <is>
           <t>no</t>
@@ -12992,16 +12736,8 @@
           <t>https://expomap.ru/expo/dacha-sad-landshaft-malaja-mehanizatsija/</t>
         </is>
       </c>
-      <c r="V108" t="inlineStr">
-        <is>
-          <t>http://dacha.interopttorg.ru/?utm_source=expomap</t>
-        </is>
-      </c>
-      <c r="W108" t="inlineStr">
-        <is>
-          <t>http://dacha.interopttorg.ru/?utm_source=expomap</t>
-        </is>
-      </c>
+      <c r="V108" t="inlineStr"/>
+      <c r="W108" t="inlineStr"/>
       <c r="X108" t="inlineStr">
         <is>
           <t>no</t>
@@ -13105,16 +12841,8 @@
           <t>https://expomap.ru/expo/edrajv/</t>
         </is>
       </c>
-      <c r="V109" t="inlineStr">
-        <is>
-          <t>https://edriveexpo.ru/</t>
-        </is>
-      </c>
-      <c r="W109" t="inlineStr">
-        <is>
-          <t>https://edriveexpo.ru/</t>
-        </is>
-      </c>
+      <c r="V109" t="inlineStr"/>
+      <c r="W109" t="inlineStr"/>
       <c r="X109" t="inlineStr">
         <is>
           <t>no</t>
@@ -13230,16 +12958,8 @@
           <t>https://expomap.ru/expo/reaktivnyj-otdyh/</t>
         </is>
       </c>
-      <c r="V110" t="inlineStr">
-        <is>
-          <t>https://activerestexpo.ru/</t>
-        </is>
-      </c>
-      <c r="W110" t="inlineStr">
-        <is>
-          <t>https://activerestexpo.ru/</t>
-        </is>
-      </c>
+      <c r="V110" t="inlineStr"/>
+      <c r="W110" t="inlineStr"/>
       <c r="X110" t="inlineStr">
         <is>
           <t>no</t>
@@ -13351,16 +13071,8 @@
           <t>https://expomap.ru/expo/motovesna/</t>
         </is>
       </c>
-      <c r="V111" t="inlineStr">
-        <is>
-          <t>https://motospring.ru/</t>
-        </is>
-      </c>
-      <c r="W111" t="inlineStr">
-        <is>
-          <t>https://motospring.ru/</t>
-        </is>
-      </c>
+      <c r="V111" t="inlineStr"/>
+      <c r="W111" t="inlineStr"/>
       <c r="X111" t="inlineStr">
         <is>
           <t>no</t>
@@ -13471,16 +13183,8 @@
           <t>https://expomap.ru/expo/velokult/</t>
         </is>
       </c>
-      <c r="V112" t="inlineStr">
-        <is>
-          <t>https://velocultexpo.ru/</t>
-        </is>
-      </c>
-      <c r="W112" t="inlineStr">
-        <is>
-          <t>https://velocultexpo.ru/</t>
-        </is>
-      </c>
+      <c r="V112" t="inlineStr"/>
+      <c r="W112" t="inlineStr"/>
       <c r="X112" t="inlineStr">
         <is>
           <t>no</t>
@@ -13687,16 +13391,8 @@
           <t>https://expomap.ru/expo/lodki-expo/2026/apr/</t>
         </is>
       </c>
-      <c r="V114" t="inlineStr">
-        <is>
-          <t>https://lodkiexpo.ru/</t>
-        </is>
-      </c>
-      <c r="W114" t="inlineStr">
-        <is>
-          <t>https://lodkiexpo.ru/</t>
-        </is>
-      </c>
+      <c r="V114" t="inlineStr"/>
+      <c r="W114" t="inlineStr"/>
       <c r="X114" t="inlineStr">
         <is>
           <t>no</t>
@@ -13801,16 +13497,8 @@
           <t>https://expomap.ru/expo/art-russia-fair/</t>
         </is>
       </c>
-      <c r="V115" t="inlineStr">
-        <is>
-          <t>https://artrussiafair.com/?ysclid=mid54tcie6399601886</t>
-        </is>
-      </c>
-      <c r="W115" t="inlineStr">
-        <is>
-          <t>https://artrussiafair.com/?ysclid=mid54tcie6399601886</t>
-        </is>
-      </c>
+      <c r="V115" t="inlineStr"/>
+      <c r="W115" t="inlineStr"/>
       <c r="X115" t="inlineStr">
         <is>
           <t>no</t>
@@ -14122,16 +13810,8 @@
           <t>https://expomap.ru/expo/portable-hi-fi-audio-show/2026/</t>
         </is>
       </c>
-      <c r="V118" t="inlineStr">
-        <is>
-          <t>https://portablehifiaudio.ru/</t>
-        </is>
-      </c>
-      <c r="W118" t="inlineStr">
-        <is>
-          <t>https://portablehifiaudio.ru/</t>
-        </is>
-      </c>
+      <c r="V118" t="inlineStr"/>
+      <c r="W118" t="inlineStr"/>
       <c r="X118" t="inlineStr">
         <is>
           <t>no</t>
@@ -14266,16 +13946,8 @@
           <t>https://expomap.ru/expo/rossijskaya-nedelya-vysokih-technologij/</t>
         </is>
       </c>
-      <c r="V119" t="inlineStr">
-        <is>
-          <t>https://hi-techweek.ru/</t>
-        </is>
-      </c>
-      <c r="W119" t="inlineStr">
-        <is>
-          <t>https://hi-techweek.ru/</t>
-        </is>
-      </c>
+      <c r="V119" t="inlineStr"/>
+      <c r="W119" t="inlineStr"/>
       <c r="X119" t="inlineStr">
         <is>
           <t>no</t>
@@ -15062,16 +14734,8 @@
           <t>https://expomap.ru/expo/krasivye-doma/</t>
         </is>
       </c>
-      <c r="V126" t="inlineStr">
-        <is>
-          <t>https://houses.ru/</t>
-        </is>
-      </c>
-      <c r="W126" t="inlineStr">
-        <is>
-          <t>https://houses.ru/</t>
-        </is>
-      </c>
+      <c r="V126" t="inlineStr"/>
+      <c r="W126" t="inlineStr"/>
       <c r="X126" t="inlineStr">
         <is>
           <t>no</t>
@@ -15338,16 +15002,8 @@
           <t>https://expomap.ru/expo/bevitec/2026/</t>
         </is>
       </c>
-      <c r="V128" t="inlineStr">
-        <is>
-          <t>https://bevitec.ru/</t>
-        </is>
-      </c>
-      <c r="W128" t="inlineStr">
-        <is>
-          <t>https://bevitec.ru/</t>
-        </is>
-      </c>
+      <c r="V128" t="inlineStr"/>
+      <c r="W128" t="inlineStr"/>
       <c r="X128" t="inlineStr">
         <is>
           <t>no</t>
@@ -15578,16 +15234,8 @@
           <t>https://expomap.ru/expo/natmallexpo/</t>
         </is>
       </c>
-      <c r="V130" t="inlineStr">
-        <is>
-          <t>https://natmall.ru/?utm_source=expomap_page&amp;utm_medium=referral&amp;utm_campaign=nm26</t>
-        </is>
-      </c>
-      <c r="W130" t="inlineStr">
-        <is>
-          <t>https://natmall.ru/?utm_source=expomap_page&amp;utm_medium=referral&amp;utm_campaign=nm26</t>
-        </is>
-      </c>
+      <c r="V130" t="inlineStr"/>
+      <c r="W130" t="inlineStr"/>
       <c r="X130" t="inlineStr">
         <is>
           <t>no</t>
@@ -16385,16 +16033,8 @@
           <t>https://expomap.ru/expo/moscow-international-property-show/</t>
         </is>
       </c>
-      <c r="V137" t="inlineStr">
-        <is>
-          <t>https://internationalproperty.ru/</t>
-        </is>
-      </c>
-      <c r="W137" t="inlineStr">
-        <is>
-          <t>https://internationalproperty.ru/</t>
-        </is>
-      </c>
+      <c r="V137" t="inlineStr"/>
+      <c r="W137" t="inlineStr"/>
       <c r="X137" t="inlineStr">
         <is>
           <t>no</t>
@@ -16510,16 +16150,8 @@
           <t>https://expomap.ru/expo/lom-chernyh-i-tsvetnyh-metallov/</t>
         </is>
       </c>
-      <c r="V138" t="inlineStr">
-        <is>
-          <t>http://lom.rusmet.ru</t>
-        </is>
-      </c>
-      <c r="W138" t="inlineStr">
-        <is>
-          <t>http://lom.rusmet.ru</t>
-        </is>
-      </c>
+      <c r="V138" t="inlineStr"/>
+      <c r="W138" t="inlineStr"/>
       <c r="X138" t="inlineStr">
         <is>
           <t>no</t>
@@ -17327,16 +16959,8 @@
           <t>https://expomap.ru/expo/dental-expo-moskva/2026/apr/</t>
         </is>
       </c>
-      <c r="V145" t="inlineStr">
-        <is>
-          <t>https://www.dental-expo.com/?format=feed&amp;type=atom</t>
-        </is>
-      </c>
-      <c r="W145" t="inlineStr">
-        <is>
-          <t>https://www.dental-expo.com/?format=feed&amp;type=atom</t>
-        </is>
-      </c>
+      <c r="V145" t="inlineStr"/>
+      <c r="W145" t="inlineStr"/>
       <c r="X145" t="inlineStr">
         <is>
           <t>no</t>
@@ -17429,16 +17053,8 @@
           <t>https://expomap.ru/expo/dental-salon-the-59th-moscow-international-dental-forum-exhibition/</t>
         </is>
       </c>
-      <c r="V146" t="inlineStr">
-        <is>
-          <t>http://en.dental-expo.com/dental-salon-en</t>
-        </is>
-      </c>
-      <c r="W146" t="inlineStr">
-        <is>
-          <t>http://en.dental-expo.com/dental-salon-en</t>
-        </is>
-      </c>
+      <c r="V146" t="inlineStr"/>
+      <c r="W146" t="inlineStr"/>
       <c r="X146" t="inlineStr">
         <is>
           <t>no</t>
@@ -18234,16 +17850,8 @@
           <t>https://expomap.ru/expo/parkseason-expo/</t>
         </is>
       </c>
-      <c r="V153" t="inlineStr">
-        <is>
-          <t>https://expo.urbanparks.ru/</t>
-        </is>
-      </c>
-      <c r="W153" t="inlineStr">
-        <is>
-          <t>https://expo.urbanparks.ru/</t>
-        </is>
-      </c>
+      <c r="V153" t="inlineStr"/>
+      <c r="W153" t="inlineStr"/>
       <c r="X153" t="inlineStr">
         <is>
           <t>no</t>
@@ -18342,16 +17950,8 @@
           <t>https://expomap.ru/expo/stsena/</t>
         </is>
       </c>
-      <c r="V154" t="inlineStr">
-        <is>
-          <t>https://clck.ru/3HPGjr</t>
-        </is>
-      </c>
-      <c r="W154" t="inlineStr">
-        <is>
-          <t>https://clck.ru/3HPGjr</t>
-        </is>
-      </c>
+      <c r="V154" t="inlineStr"/>
+      <c r="W154" t="inlineStr"/>
       <c r="X154" t="inlineStr">
         <is>
           <t>no</t>
@@ -18566,16 +18166,8 @@
           <t>https://expomap.ru/expo/psycoach-expo/2026/apr/</t>
         </is>
       </c>
-      <c r="V156" t="inlineStr">
-        <is>
-          <t>https://psycoach-expo.ru/</t>
-        </is>
-      </c>
-      <c r="W156" t="inlineStr">
-        <is>
-          <t>https://psycoach-expo.ru/</t>
-        </is>
-      </c>
+      <c r="V156" t="inlineStr"/>
+      <c r="W156" t="inlineStr"/>
       <c r="X156" t="inlineStr">
         <is>
           <t>no</t>
@@ -19338,16 +18930,8 @@
           <t>https://expomap.ru/expo/premiya-beauty-awards/2026/</t>
         </is>
       </c>
-      <c r="V163" t="inlineStr">
-        <is>
-          <t>https://beauty-awards.ru</t>
-        </is>
-      </c>
-      <c r="W163" t="inlineStr">
-        <is>
-          <t>https://beauty-awards.ru</t>
-        </is>
-      </c>
+      <c r="V163" t="inlineStr"/>
+      <c r="W163" t="inlineStr"/>
       <c r="X163" t="inlineStr">
         <is>
           <t>no</t>
@@ -19809,16 +19393,8 @@
           <t>https://expomap.ru/expo/goszakaz/</t>
         </is>
       </c>
-      <c r="V167" t="inlineStr">
-        <is>
-          <t>https://forum-goszakaz.ru/</t>
-        </is>
-      </c>
-      <c r="W167" t="inlineStr">
-        <is>
-          <t>https://forum-goszakaz.ru/</t>
-        </is>
-      </c>
+      <c r="V167" t="inlineStr"/>
+      <c r="W167" t="inlineStr"/>
       <c r="X167" t="inlineStr">
         <is>
           <t>no</t>
@@ -20149,16 +19725,8 @@
           <t>https://expomap.ru/expo/konnaja/</t>
         </is>
       </c>
-      <c r="V170" t="inlineStr">
-        <is>
-          <t>http://equinerussia.ru/</t>
-        </is>
-      </c>
-      <c r="W170" t="inlineStr">
-        <is>
-          <t>http://equinerussia.ru/</t>
-        </is>
-      </c>
+      <c r="V170" t="inlineStr"/>
+      <c r="W170" t="inlineStr"/>
       <c r="X170" t="inlineStr">
         <is>
           <t>no</t>
@@ -20269,16 +19837,8 @@
           <t>https://expomap.ru/expo/refcold-russia/</t>
         </is>
       </c>
-      <c r="V171" t="inlineStr">
-        <is>
-          <t>https://holodexpo.ru/</t>
-        </is>
-      </c>
-      <c r="W171" t="inlineStr">
-        <is>
-          <t>https://holodexpo.ru/</t>
-        </is>
-      </c>
+      <c r="V171" t="inlineStr"/>
+      <c r="W171" t="inlineStr"/>
       <c r="X171" t="inlineStr">
         <is>
           <t>no</t>
@@ -20636,16 +20196,8 @@
           <t>https://expomap.ru/expo/teplo-i-energetika-heat-electro/</t>
         </is>
       </c>
-      <c r="V174" t="inlineStr">
-        <is>
-          <t>https://www.machinery-fair.ru/</t>
-        </is>
-      </c>
-      <c r="W174" t="inlineStr">
-        <is>
-          <t>https://www.machinery-fair.ru/</t>
-        </is>
-      </c>
+      <c r="V174" t="inlineStr"/>
+      <c r="W174" t="inlineStr"/>
       <c r="X174" t="inlineStr">
         <is>
           <t>no</t>
@@ -20865,16 +20417,8 @@
           <t>https://expomap.ru/expo/mice-excellence-awards/</t>
         </is>
       </c>
-      <c r="V176" t="inlineStr">
-        <is>
-          <t>https://mice-awards.com/#subscribe</t>
-        </is>
-      </c>
-      <c r="W176" t="inlineStr">
-        <is>
-          <t>https://mice-awards.com/#subscribe</t>
-        </is>
-      </c>
+      <c r="V176" t="inlineStr"/>
+      <c r="W176" t="inlineStr"/>
       <c r="X176" t="inlineStr">
         <is>
           <t>no</t>
@@ -20971,16 +20515,8 @@
           <t>https://expomap.ru/expo/russian-grill-fest/</t>
         </is>
       </c>
-      <c r="V177" t="inlineStr">
-        <is>
-          <t>https://russiangrillfest.ru</t>
-        </is>
-      </c>
-      <c r="W177" t="inlineStr">
-        <is>
-          <t>https://russiangrillfest.ru</t>
-        </is>
-      </c>
+      <c r="V177" t="inlineStr"/>
+      <c r="W177" t="inlineStr"/>
       <c r="X177" t="inlineStr">
         <is>
           <t>no</t>
@@ -21302,16 +20838,8 @@
           <t>https://expomap.ru/expo/meditsinskaja-diagnostika/</t>
         </is>
       </c>
-      <c r="V180" t="inlineStr">
-        <is>
-          <t>https://www.mediexpo.ru/calendar/forums/med-2026/index/</t>
-        </is>
-      </c>
-      <c r="W180" t="inlineStr">
-        <is>
-          <t>https://www.mediexpo.ru/calendar/forums/med-2026/index/</t>
-        </is>
-      </c>
+      <c r="V180" t="inlineStr"/>
+      <c r="W180" t="inlineStr"/>
       <c r="X180" t="inlineStr">
         <is>
           <t>no</t>
@@ -21660,16 +21188,8 @@
           <t>https://expomap.ru/expo/metallokonstruktsii/</t>
         </is>
       </c>
-      <c r="V183" t="inlineStr">
-        <is>
-          <t>https://mc-expo.ru/en</t>
-        </is>
-      </c>
-      <c r="W183" t="inlineStr">
-        <is>
-          <t>https://mc-expo.ru/en</t>
-        </is>
-      </c>
+      <c r="V183" t="inlineStr"/>
+      <c r="W183" t="inlineStr"/>
       <c r="X183" t="inlineStr">
         <is>
           <t>no</t>
@@ -21770,16 +21290,8 @@
           <t>https://expomap.ru/expo/stt-expo/2026/</t>
         </is>
       </c>
-      <c r="V184" t="inlineStr">
-        <is>
-          <t>https://www.ctt-expo.ru/</t>
-        </is>
-      </c>
-      <c r="W184" t="inlineStr">
-        <is>
-          <t>https://www.ctt-expo.ru/</t>
-        </is>
-      </c>
+      <c r="V184" t="inlineStr"/>
+      <c r="W184" t="inlineStr"/>
       <c r="X184" t="inlineStr">
         <is>
           <t>no</t>
@@ -21903,16 +21415,8 @@
           <t>https://expomap.ru/expo/ctt-expo/</t>
         </is>
       </c>
-      <c r="V185" t="inlineStr">
-        <is>
-          <t>https://ctt-expo.ru/about-eng</t>
-        </is>
-      </c>
-      <c r="W185" t="inlineStr">
-        <is>
-          <t>https://ctt-expo.ru/about-eng</t>
-        </is>
-      </c>
+      <c r="V185" t="inlineStr"/>
+      <c r="W185" t="inlineStr"/>
       <c r="X185" t="inlineStr">
         <is>
           <t>no</t>
@@ -22017,16 +21521,8 @@
           <t>https://expomap.ru/expo/sto-expo/</t>
         </is>
       </c>
-      <c r="V186" t="inlineStr">
-        <is>
-          <t>https://www.cto-expo.ru/</t>
-        </is>
-      </c>
-      <c r="W186" t="inlineStr">
-        <is>
-          <t>https://www.cto-expo.ru/</t>
-        </is>
-      </c>
+      <c r="V186" t="inlineStr"/>
+      <c r="W186" t="inlineStr"/>
       <c r="X186" t="inlineStr">
         <is>
           <t>no</t>
@@ -22138,16 +21634,8 @@
           <t>https://expomap.ru/expo/logistika-expo/</t>
         </is>
       </c>
-      <c r="V187" t="inlineStr">
-        <is>
-          <t>https://logistika-expo.ru/</t>
-        </is>
-      </c>
-      <c r="W187" t="inlineStr">
-        <is>
-          <t>https://logistika-expo.ru/</t>
-        </is>
-      </c>
+      <c r="V187" t="inlineStr"/>
+      <c r="W187" t="inlineStr"/>
       <c r="X187" t="inlineStr">
         <is>
           <t>no</t>
@@ -22365,16 +21853,8 @@
           <t>https://expomap.ru/expo/seller-fest/</t>
         </is>
       </c>
-      <c r="V189" t="inlineStr">
-        <is>
-          <t>https://sellerfest.ru/sellerfest.ru</t>
-        </is>
-      </c>
-      <c r="W189" t="inlineStr">
-        <is>
-          <t>https://sellerfest.ru/sellerfest.ru</t>
-        </is>
-      </c>
+      <c r="V189" t="inlineStr"/>
+      <c r="W189" t="inlineStr"/>
       <c r="X189" t="inlineStr">
         <is>
           <t>no</t>
@@ -22493,16 +21973,8 @@
           <t>https://expomap.ru/expo/nachalnaja-voennaja-podgotovka/</t>
         </is>
       </c>
-      <c r="V190" t="inlineStr">
-        <is>
-          <t>https://nvpexpo.ru/</t>
-        </is>
-      </c>
-      <c r="W190" t="inlineStr">
-        <is>
-          <t>https://nvpexpo.ru/</t>
-        </is>
-      </c>
+      <c r="V190" t="inlineStr"/>
+      <c r="W190" t="inlineStr"/>
       <c r="X190" t="inlineStr">
         <is>
           <t>no</t>
@@ -22615,16 +22087,8 @@
           <t>https://expomap.ru/expo/ekipirovka/</t>
         </is>
       </c>
-      <c r="V191" t="inlineStr">
-        <is>
-          <t>https://equipexpo.ru/</t>
-        </is>
-      </c>
-      <c r="W191" t="inlineStr">
-        <is>
-          <t>https://equipexpo.ru/</t>
-        </is>
-      </c>
+      <c r="V191" t="inlineStr"/>
+      <c r="W191" t="inlineStr"/>
       <c r="X191" t="inlineStr">
         <is>
           <t>no</t>
@@ -22734,16 +22198,8 @@
           <t>https://expomap.ru/expo/arh-moskva/</t>
         </is>
       </c>
-      <c r="V192" t="inlineStr">
-        <is>
-          <t>https://www.archmoscow.ru/</t>
-        </is>
-      </c>
-      <c r="W192" t="inlineStr">
-        <is>
-          <t>https://www.archmoscow.ru/</t>
-        </is>
-      </c>
+      <c r="V192" t="inlineStr"/>
+      <c r="W192" t="inlineStr"/>
       <c r="X192" t="inlineStr">
         <is>
           <t>no</t>
@@ -22849,16 +22305,8 @@
           <t>https://expomap.ru/expo/next-home/</t>
         </is>
       </c>
-      <c r="V193" t="inlineStr">
-        <is>
-          <t>https://forum-nexthome.ru/?ysclid=miirwte46m91445796</t>
-        </is>
-      </c>
-      <c r="W193" t="inlineStr">
-        <is>
-          <t>https://forum-nexthome.ru/?ysclid=miirwte46m91445796</t>
-        </is>
-      </c>
+      <c r="V193" t="inlineStr"/>
+      <c r="W193" t="inlineStr"/>
       <c r="X193" t="inlineStr">
         <is>
           <t>no</t>
@@ -23304,16 +22752,8 @@
           <t>https://expomap.ru/expo/sakvoyazh/2026/jun/</t>
         </is>
       </c>
-      <c r="V197" t="inlineStr">
-        <is>
-          <t>https://sakvoyazhlife.ru/</t>
-        </is>
-      </c>
-      <c r="W197" t="inlineStr">
-        <is>
-          <t>https://sakvoyazhlife.ru/</t>
-        </is>
-      </c>
+      <c r="V197" t="inlineStr"/>
+      <c r="W197" t="inlineStr"/>
       <c r="X197" t="inlineStr">
         <is>
           <t>no</t>
@@ -23643,16 +23083,8 @@
           <t>https://expomap.ru/expo/rosmould-3d-tech-jun/2026/</t>
         </is>
       </c>
-      <c r="V200" t="inlineStr">
-        <is>
-          <t>https://rosmould.ru/</t>
-        </is>
-      </c>
-      <c r="W200" t="inlineStr">
-        <is>
-          <t>https://rosmould.ru/</t>
-        </is>
-      </c>
+      <c r="V200" t="inlineStr"/>
+      <c r="W200" t="inlineStr"/>
       <c r="X200" t="inlineStr">
         <is>
           <t>no</t>
@@ -23780,16 +23212,8 @@
           <t>https://expomap.ru/expo/technotekstil-technokompozit-technopolimer/</t>
         </is>
       </c>
-      <c r="V201" t="inlineStr">
-        <is>
-          <t>https://tech-textile.ru/?ysclid=mgkoblrveu489153325</t>
-        </is>
-      </c>
-      <c r="W201" t="inlineStr">
-        <is>
-          <t>https://tech-textile.ru/?ysclid=mgkoblrveu489153325</t>
-        </is>
-      </c>
+      <c r="V201" t="inlineStr"/>
+      <c r="W201" t="inlineStr"/>
       <c r="X201" t="inlineStr">
         <is>
           <t>no</t>
@@ -23905,16 +23329,8 @@
           <t>https://expomap.ru/expo/rosplast/</t>
         </is>
       </c>
-      <c r="V202" t="inlineStr">
-        <is>
-          <t>https://rosplast-expo.ru/</t>
-        </is>
-      </c>
-      <c r="W202" t="inlineStr">
-        <is>
-          <t>https://rosplast-expo.ru/</t>
-        </is>
-      </c>
+      <c r="V202" t="inlineStr"/>
+      <c r="W202" t="inlineStr"/>
       <c r="X202" t="inlineStr">
         <is>
           <t>no</t>
@@ -24025,16 +23441,8 @@
           <t>https://expomap.ru/expo/3d-tech-by-rosmould/</t>
         </is>
       </c>
-      <c r="V203" t="inlineStr">
-        <is>
-          <t>https://3dtech-expo.ru/</t>
-        </is>
-      </c>
-      <c r="W203" t="inlineStr">
-        <is>
-          <t>https://3dtech-expo.ru/</t>
-        </is>
-      </c>
+      <c r="V203" t="inlineStr"/>
+      <c r="W203" t="inlineStr"/>
       <c r="X203" t="inlineStr">
         <is>
           <t>no</t>
@@ -24268,16 +23676,8 @@
           <t>https://expomap.ru/expo/rosmould-3d-tech/</t>
         </is>
       </c>
-      <c r="V205" t="inlineStr">
-        <is>
-          <t>https://rosmould.ru/</t>
-        </is>
-      </c>
-      <c r="W205" t="inlineStr">
-        <is>
-          <t>https://rosmould.ru/</t>
-        </is>
-      </c>
+      <c r="V205" t="inlineStr"/>
+      <c r="W205" t="inlineStr"/>
       <c r="X205" t="inlineStr">
         <is>
           <t>no</t>
@@ -24514,16 +23914,8 @@
           <t>https://expomap.ru/expo/sptokrany/</t>
         </is>
       </c>
-      <c r="V207" t="inlineStr">
-        <is>
-          <t>https://www.crane-expo.ru</t>
-        </is>
-      </c>
-      <c r="W207" t="inlineStr">
-        <is>
-          <t>https://www.crane-expo.ru</t>
-        </is>
-      </c>
+      <c r="V207" t="inlineStr"/>
+      <c r="W207" t="inlineStr"/>
       <c r="X207" t="inlineStr">
         <is>
           <t>no</t>
@@ -24730,16 +24122,8 @@
           <t>https://expomap.ru/expo/wowbiz/</t>
         </is>
       </c>
-      <c r="V209" t="inlineStr">
-        <is>
-          <t>https://wowbiz.global/</t>
-        </is>
-      </c>
-      <c r="W209" t="inlineStr">
-        <is>
-          <t>https://wowbiz.global/</t>
-        </is>
-      </c>
+      <c r="V209" t="inlineStr"/>
+      <c r="W209" t="inlineStr"/>
       <c r="X209" t="inlineStr">
         <is>
           <t>no</t>
@@ -24844,16 +24228,8 @@
           <t>https://expomap.ru/expo/reindustry-expo/2026/</t>
         </is>
       </c>
-      <c r="V210" t="inlineStr">
-        <is>
-          <t>https://reindustry-expo.ru/</t>
-        </is>
-      </c>
-      <c r="W210" t="inlineStr">
-        <is>
-          <t>https://reindustry-expo.ru/</t>
-        </is>
-      </c>
+      <c r="V210" t="inlineStr"/>
+      <c r="W210" t="inlineStr"/>
       <c r="X210" t="inlineStr">
         <is>
           <t>no</t>
@@ -25438,16 +24814,8 @@
           <t>https://expomap.ru/expo/media-menedzher-rossii/</t>
         </is>
       </c>
-      <c r="V215" t="inlineStr">
-        <is>
-          <t>https://www.media-manager.ru/</t>
-        </is>
-      </c>
-      <c r="W215" t="inlineStr">
-        <is>
-          <t>https://www.media-manager.ru/</t>
-        </is>
-      </c>
+      <c r="V215" t="inlineStr"/>
+      <c r="W215" t="inlineStr"/>
       <c r="X215" t="inlineStr">
         <is>
           <t>no</t>
@@ -25555,16 +24923,8 @@
           <t>https://expomap.ru/expo/epiccon-russia-moskva/</t>
         </is>
       </c>
-      <c r="V216" t="inlineStr">
-        <is>
-          <t>https://epiccon.ru/</t>
-        </is>
-      </c>
-      <c r="W216" t="inlineStr">
-        <is>
-          <t>https://epiccon.ru/</t>
-        </is>
-      </c>
+      <c r="V216" t="inlineStr"/>
+      <c r="W216" t="inlineStr"/>
       <c r="X216" t="inlineStr">
         <is>
           <t>no</t>
@@ -25869,16 +25229,8 @@
           <t>https://expomap.ru/expo/den-polya-moskovskoj-oblasti/</t>
         </is>
       </c>
-      <c r="V219" t="inlineStr">
-        <is>
-          <t>https://pole50.ru/</t>
-        </is>
-      </c>
-      <c r="W219" t="inlineStr">
-        <is>
-          <t>https://pole50.ru/</t>
-        </is>
-      </c>
+      <c r="V219" t="inlineStr"/>
+      <c r="W219" t="inlineStr"/>
       <c r="X219" t="inlineStr">
         <is>
           <t>no</t>
@@ -26601,16 +25953,8 @@
           <t>https://expomap.ru/expo/technologii-voennoj-meditsiny-i-reabilitatsii/</t>
         </is>
       </c>
-      <c r="V225" t="inlineStr">
-        <is>
-          <t>https://vphexpo.ru/</t>
-        </is>
-      </c>
-      <c r="W225" t="inlineStr">
-        <is>
-          <t>https://vphexpo.ru/</t>
-        </is>
-      </c>
+      <c r="V225" t="inlineStr"/>
+      <c r="W225" t="inlineStr"/>
       <c r="X225" t="inlineStr">
         <is>
           <t>no</t>
@@ -27069,16 +26413,8 @@
           <t>https://expomap.ru/expo/china-commodity-fair/</t>
         </is>
       </c>
-      <c r="V229" t="inlineStr">
-        <is>
-          <t>http://en.icf-expo.ru</t>
-        </is>
-      </c>
-      <c r="W229" t="inlineStr">
-        <is>
-          <t>http://en.icf-expo.ru</t>
-        </is>
-      </c>
+      <c r="V229" t="inlineStr"/>
+      <c r="W229" t="inlineStr"/>
       <c r="X229" t="inlineStr">
         <is>
           <t>no</t>
@@ -27414,16 +26750,8 @@
           <t>https://expomap.ru/expo/home-estate-expo-vystavka-novostroek/</t>
         </is>
       </c>
-      <c r="V232" t="inlineStr">
-        <is>
-          <t>https://home-estate-expo.ru/</t>
-        </is>
-      </c>
-      <c r="W232" t="inlineStr">
-        <is>
-          <t>https://home-estate-expo.ru/</t>
-        </is>
-      </c>
+      <c r="V232" t="inlineStr"/>
+      <c r="W232" t="inlineStr"/>
       <c r="X232" t="inlineStr">
         <is>
           <t>no</t>
@@ -27547,16 +26875,8 @@
           <t>https://expomap.ru/expo/cpm-collection-premiere-moscow/</t>
         </is>
       </c>
-      <c r="V233" t="inlineStr">
-        <is>
-          <t>https://cpm-moscow.com/?lang=ru/?erid=2VfnxyWEqvi</t>
-        </is>
-      </c>
-      <c r="W233" t="inlineStr">
-        <is>
-          <t>https://cpm-moscow.com/?lang=ru/?erid=2VfnxyWEqvi</t>
-        </is>
-      </c>
+      <c r="V233" t="inlineStr"/>
+      <c r="W233" t="inlineStr"/>
       <c r="X233" t="inlineStr">
         <is>
           <t>no</t>
@@ -27674,16 +26994,8 @@
           <t>https://expomap.ru/expo/dreams-by-cpm/</t>
         </is>
       </c>
-      <c r="V234" t="inlineStr">
-        <is>
-          <t>https://dreams-moscow.com/?lang=ru/?erid=2VfnxwmRgmG</t>
-        </is>
-      </c>
-      <c r="W234" t="inlineStr">
-        <is>
-          <t>https://dreams-moscow.com/?lang=ru/?erid=2VfnxwmRgmG</t>
-        </is>
-      </c>
+      <c r="V234" t="inlineStr"/>
+      <c r="W234" t="inlineStr"/>
       <c r="X234" t="inlineStr">
         <is>
           <t>no</t>
@@ -27807,16 +27119,8 @@
           <t>https://expomap.ru/expo/otdyh-leisure/</t>
         </is>
       </c>
-      <c r="V235" t="inlineStr">
-        <is>
-          <t>https://tourismexpo.ru/?erid=2VfnxxBd5eq</t>
-        </is>
-      </c>
-      <c r="W235" t="inlineStr">
-        <is>
-          <t>https://tourismexpo.ru/?erid=2VfnxxBd5eq</t>
-        </is>
-      </c>
+      <c r="V235" t="inlineStr"/>
+      <c r="W235" t="inlineStr"/>
       <c r="X235" t="inlineStr">
         <is>
           <t>no</t>
@@ -27929,16 +27233,8 @@
           <t>https://expomap.ru/expo/textile-salon/</t>
         </is>
       </c>
-      <c r="V236" t="inlineStr">
-        <is>
-          <t>https://textile-salon.ru/</t>
-        </is>
-      </c>
-      <c r="W236" t="inlineStr">
-        <is>
-          <t>https://textile-salon.ru/</t>
-        </is>
-      </c>
+      <c r="V236" t="inlineStr"/>
+      <c r="W236" t="inlineStr"/>
       <c r="X236" t="inlineStr">
         <is>
           <t>no</t>
@@ -28038,16 +27334,8 @@
           <t>https://expomap.ru/expo/forum-dlya-proav-i-it-specialistov/2026/sep/</t>
         </is>
       </c>
-      <c r="V237" t="inlineStr">
-        <is>
-          <t>https://www.avclub.pro/event/avfocus26moskva/</t>
-        </is>
-      </c>
-      <c r="W237" t="inlineStr">
-        <is>
-          <t>https://www.avclub.pro/event/avfocus26moskva/</t>
-        </is>
-      </c>
+      <c r="V237" t="inlineStr"/>
+      <c r="W237" t="inlineStr"/>
       <c r="X237" t="inlineStr">
         <is>
           <t>no</t>
@@ -28296,16 +27584,8 @@
           <t>https://expomap.ru/expo/flowersexpo-tsvetyexpo/</t>
         </is>
       </c>
-      <c r="V239" t="inlineStr">
-        <is>
-          <t>https://www.flowers-expo.ru/</t>
-        </is>
-      </c>
-      <c r="W239" t="inlineStr">
-        <is>
-          <t>https://www.flowers-expo.ru/</t>
-        </is>
-      </c>
+      <c r="V239" t="inlineStr"/>
+      <c r="W239" t="inlineStr"/>
       <c r="X239" t="inlineStr">
         <is>
           <t>no</t>
@@ -28398,16 +27678,8 @@
           <t>https://expomap.ru/expo/flowers-expo/</t>
         </is>
       </c>
-      <c r="V240" t="inlineStr">
-        <is>
-          <t>http://www.flowers-expo.ru</t>
-        </is>
-      </c>
-      <c r="W240" t="inlineStr">
-        <is>
-          <t>http://www.flowers-expo.ru</t>
-        </is>
-      </c>
+      <c r="V240" t="inlineStr"/>
+      <c r="W240" t="inlineStr"/>
       <c r="X240" t="inlineStr">
         <is>
           <t>no</t>
@@ -29113,16 +28385,8 @@
           <t>https://expomap.ru/expo/sekrety-otelera-moskva/</t>
         </is>
       </c>
-      <c r="V246" t="inlineStr">
-        <is>
-          <t>https://hoteliersecret.pro/moscow</t>
-        </is>
-      </c>
-      <c r="W246" t="inlineStr">
-        <is>
-          <t>https://hoteliersecret.pro/moscow</t>
-        </is>
-      </c>
+      <c r="V246" t="inlineStr"/>
+      <c r="W246" t="inlineStr"/>
       <c r="X246" t="inlineStr">
         <is>
           <t>no</t>
@@ -29231,16 +28495,8 @@
           <t>https://expomap.ru/expo/sitipajp/</t>
         </is>
       </c>
-      <c r="V247" t="inlineStr">
-        <is>
-          <t>https://ecwatech.ru/citypipe</t>
-        </is>
-      </c>
-      <c r="W247" t="inlineStr">
-        <is>
-          <t>https://ecwatech.ru/citypipe</t>
-        </is>
-      </c>
+      <c r="V247" t="inlineStr"/>
+      <c r="W247" t="inlineStr"/>
       <c r="X247" t="inlineStr">
         <is>
           <t>no</t>
@@ -29350,16 +28606,8 @@
           <t>https://expomap.ru/expo/no-dig-moskva/</t>
         </is>
       </c>
-      <c r="V248" t="inlineStr">
-        <is>
-          <t>https://ecwatech.ru/nodig</t>
-        </is>
-      </c>
-      <c r="W248" t="inlineStr">
-        <is>
-          <t>https://ecwatech.ru/nodig</t>
-        </is>
-      </c>
+      <c r="V248" t="inlineStr"/>
+      <c r="W248" t="inlineStr"/>
       <c r="X248" t="inlineStr">
         <is>
           <t>no</t>
@@ -29487,16 +28735,8 @@
           <t>https://expomap.ru/expo/worldfood-moscow/</t>
         </is>
       </c>
-      <c r="V249" t="inlineStr">
-        <is>
-          <t>https://expoworldfood.com/?erid=2VfnxyRv47s</t>
-        </is>
-      </c>
-      <c r="W249" t="inlineStr">
-        <is>
-          <t>https://expoworldfood.com/?erid=2VfnxyRv47s</t>
-        </is>
-      </c>
+      <c r="V249" t="inlineStr"/>
+      <c r="W249" t="inlineStr"/>
       <c r="X249" t="inlineStr">
         <is>
           <t>no</t>
@@ -29730,16 +28970,8 @@
           <t>https://expomap.ru/expo/tekstillegprom/</t>
         </is>
       </c>
-      <c r="V251" t="inlineStr">
-        <is>
-          <t>https://textilexpo.ru/</t>
-        </is>
-      </c>
-      <c r="W251" t="inlineStr">
-        <is>
-          <t>https://textilexpo.ru/</t>
-        </is>
-      </c>
+      <c r="V251" t="inlineStr"/>
+      <c r="W251" t="inlineStr"/>
       <c r="X251" t="inlineStr">
         <is>
           <t>no</t>
@@ -29963,16 +29195,8 @@
           <t>https://expomap.ru/expo/teploenergetika-rossii-stroitelstvo-i-modernizatsija-stantsij/</t>
         </is>
       </c>
-      <c r="V253" t="inlineStr">
-        <is>
-          <t>https://www.thermalpowerrussia.ru/?utm_source=expomap</t>
-        </is>
-      </c>
-      <c r="W253" t="inlineStr">
-        <is>
-          <t>https://www.thermalpowerrussia.ru/?utm_source=expomap</t>
-        </is>
-      </c>
+      <c r="V253" t="inlineStr"/>
+      <c r="W253" t="inlineStr"/>
       <c r="X253" t="inlineStr">
         <is>
           <t>no</t>
@@ -30434,16 +29658,8 @@
           <t>https://expomap.ru/expo/design/</t>
         </is>
       </c>
-      <c r="V257" t="inlineStr">
-        <is>
-          <t>https://design-plus.ru/</t>
-        </is>
-      </c>
-      <c r="W257" t="inlineStr">
-        <is>
-          <t>https://design-plus.ru/</t>
-        </is>
-      </c>
+      <c r="V257" t="inlineStr"/>
+      <c r="W257" t="inlineStr"/>
       <c r="X257" t="inlineStr">
         <is>
           <t>no</t>
@@ -30553,16 +29769,8 @@
           <t>https://expomap.ru/expo/homefest/</t>
         </is>
       </c>
-      <c r="V258" t="inlineStr">
-        <is>
-          <t>https://homefest.ru/</t>
-        </is>
-      </c>
-      <c r="W258" t="inlineStr">
-        <is>
-          <t>https://homefest.ru/</t>
-        </is>
-      </c>
+      <c r="V258" t="inlineStr"/>
+      <c r="W258" t="inlineStr"/>
       <c r="X258" t="inlineStr">
         <is>
           <t>no</t>
@@ -30655,16 +29863,8 @@
           <t>https://expomap.ru/expo/dental-expo-the-60th-moscow-international-dental-forum-exhibition/</t>
         </is>
       </c>
-      <c r="V259" t="inlineStr">
-        <is>
-          <t>http://en.dental-expo.com/dental-expo-en</t>
-        </is>
-      </c>
-      <c r="W259" t="inlineStr">
-        <is>
-          <t>http://en.dental-expo.com/dental-expo-en</t>
-        </is>
-      </c>
+      <c r="V259" t="inlineStr"/>
+      <c r="W259" t="inlineStr"/>
       <c r="X259" t="inlineStr">
         <is>
           <t>no</t>
@@ -30911,16 +30111,8 @@
           <t>https://expomap.ru/expo/parkzoo/</t>
         </is>
       </c>
-      <c r="V261" t="inlineStr">
-        <is>
-          <t>https://www.parkzoo.ru/</t>
-        </is>
-      </c>
-      <c r="W261" t="inlineStr">
-        <is>
-          <t>https://www.parkzoo.ru/</t>
-        </is>
-      </c>
+      <c r="V261" t="inlineStr"/>
+      <c r="W261" t="inlineStr"/>
       <c r="X261" t="inlineStr">
         <is>
           <t>no</t>
@@ -31156,16 +30348,8 @@
           <t>https://expomap.ru/expo/mir-ohoty-i-rybalki/2026/sep/</t>
         </is>
       </c>
-      <c r="V263" t="inlineStr">
-        <is>
-          <t>https://www.huntfishexpo.ru/</t>
-        </is>
-      </c>
-      <c r="W263" t="inlineStr">
-        <is>
-          <t>https://www.huntfishexpo.ru/</t>
-        </is>
-      </c>
+      <c r="V263" t="inlineStr"/>
+      <c r="W263" t="inlineStr"/>
       <c r="X263" t="inlineStr">
         <is>
           <t>no</t>
@@ -31270,16 +30454,8 @@
           <t>https://expomap.ru/expo/muzhskoe-zdorove-i-dolgoletie/</t>
         </is>
       </c>
-      <c r="V264" t="inlineStr">
-        <is>
-          <t>https://qlm-expo.ru/</t>
-        </is>
-      </c>
-      <c r="W264" t="inlineStr">
-        <is>
-          <t>https://qlm-expo.ru/</t>
-        </is>
-      </c>
+      <c r="V264" t="inlineStr"/>
+      <c r="W264" t="inlineStr"/>
       <c r="X264" t="inlineStr">
         <is>
           <t>no</t>
@@ -31389,16 +30565,8 @@
           <t>https://expomap.ru/expo/eco-beauty-expo/</t>
         </is>
       </c>
-      <c r="V265" t="inlineStr">
-        <is>
-          <t>https://eco-beauty-expo.ru/?ysclid=mpfcu5eekb658205766</t>
-        </is>
-      </c>
-      <c r="W265" t="inlineStr">
-        <is>
-          <t>https://eco-beauty-expo.ru/?ysclid=mpfcu5eekb658205766</t>
-        </is>
-      </c>
+      <c r="V265" t="inlineStr"/>
+      <c r="W265" t="inlineStr"/>
       <c r="X265" t="inlineStr">
         <is>
           <t>no</t>
@@ -31516,16 +30684,8 @@
           <t>https://expomap.ru/expo/makeup-expo/</t>
         </is>
       </c>
-      <c r="V266" t="inlineStr">
-        <is>
-          <t>https://makeup-expo.ru/?utm_source=expomap</t>
-        </is>
-      </c>
-      <c r="W266" t="inlineStr">
-        <is>
-          <t>https://makeup-expo.ru/?utm_source=expomap</t>
-        </is>
-      </c>
+      <c r="V266" t="inlineStr"/>
+      <c r="W266" t="inlineStr"/>
       <c r="X266" t="inlineStr">
         <is>
           <t>no</t>
@@ -31643,16 +30803,8 @@
           <t>https://expomap.ru/expo/healthy-hair-expo/</t>
         </is>
       </c>
-      <c r="V267" t="inlineStr">
-        <is>
-          <t>https://healthy-hair-expo.ru/?utm_source=expomap</t>
-        </is>
-      </c>
-      <c r="W267" t="inlineStr">
-        <is>
-          <t>https://healthy-hair-expo.ru/?utm_source=expomap</t>
-        </is>
-      </c>
+      <c r="V267" t="inlineStr"/>
+      <c r="W267" t="inlineStr"/>
       <c r="X267" t="inlineStr">
         <is>
           <t>no</t>
@@ -31778,16 +30930,8 @@
           <t>https://expomap.ru/expo/zozh-expo/</t>
         </is>
       </c>
-      <c r="V268" t="inlineStr">
-        <is>
-          <t>https://zozhexpo.ru/</t>
-        </is>
-      </c>
-      <c r="W268" t="inlineStr">
-        <is>
-          <t>https://zozhexpo.ru/</t>
-        </is>
-      </c>
+      <c r="V268" t="inlineStr"/>
+      <c r="W268" t="inlineStr"/>
       <c r="X268" t="inlineStr">
         <is>
           <t>no</t>
@@ -31907,16 +31051,8 @@
           <t>https://expomap.ru/expo/agroprodmash/</t>
         </is>
       </c>
-      <c r="V269" t="inlineStr">
-        <is>
-          <t>https://www.agroprodmash-expo.ru/</t>
-        </is>
-      </c>
-      <c r="W269" t="inlineStr">
-        <is>
-          <t>https://www.agroprodmash-expo.ru/</t>
-        </is>
-      </c>
+      <c r="V269" t="inlineStr"/>
+      <c r="W269" t="inlineStr"/>
       <c r="X269" t="inlineStr">
         <is>
           <t>no</t>
@@ -32034,16 +31170,8 @@
           <t>https://expomap.ru/expo/apteka/</t>
         </is>
       </c>
-      <c r="V270" t="inlineStr">
-        <is>
-          <t>https://aptekaexpo.ru/?erid=2VfnxveUQbj</t>
-        </is>
-      </c>
-      <c r="W270" t="inlineStr">
-        <is>
-          <t>https://aptekaexpo.ru/?erid=2VfnxveUQbj</t>
-        </is>
-      </c>
+      <c r="V270" t="inlineStr"/>
+      <c r="W270" t="inlineStr"/>
       <c r="X270" t="inlineStr">
         <is>
           <t>no</t>
@@ -32160,16 +31288,8 @@
           <t>https://expomap.ru/expo/citybus/</t>
         </is>
       </c>
-      <c r="V271" t="inlineStr">
-        <is>
-          <t>https://citybus-expo.ru/</t>
-        </is>
-      </c>
-      <c r="W271" t="inlineStr">
-        <is>
-          <t>https://citybus-expo.ru/</t>
-        </is>
-      </c>
+      <c r="V271" t="inlineStr"/>
+      <c r="W271" t="inlineStr"/>
       <c r="X271" t="inlineStr">
         <is>
           <t>no</t>
@@ -32535,16 +31655,8 @@
           <t>https://expomap.ru/expo/elektronika-transport/</t>
         </is>
       </c>
-      <c r="V274" t="inlineStr">
-        <is>
-          <t>https://e-transport.ru/</t>
-        </is>
-      </c>
-      <c r="W274" t="inlineStr">
-        <is>
-          <t>https://e-transport.ru/</t>
-        </is>
-      </c>
+      <c r="V274" t="inlineStr"/>
+      <c r="W274" t="inlineStr"/>
       <c r="X274" t="inlineStr">
         <is>
           <t>no</t>
@@ -32670,16 +31782,8 @@
           <t>https://expomap.ru/expo/intertkan/</t>
         </is>
       </c>
-      <c r="V275" t="inlineStr">
-        <is>
-          <t>https://intertkan.ru/</t>
-        </is>
-      </c>
-      <c r="W275" t="inlineStr">
-        <is>
-          <t>https://intertkan.ru/</t>
-        </is>
-      </c>
+      <c r="V275" t="inlineStr"/>
+      <c r="W275" t="inlineStr"/>
       <c r="X275" t="inlineStr">
         <is>
           <t>no</t>
@@ -32798,16 +31902,8 @@
           <t>https://expomap.ru/expo/elektrotrans/</t>
         </is>
       </c>
-      <c r="V276" t="inlineStr">
-        <is>
-          <t>https://electrotrans-expo.ru/</t>
-        </is>
-      </c>
-      <c r="W276" t="inlineStr">
-        <is>
-          <t>https://electrotrans-expo.ru/</t>
-        </is>
-      </c>
+      <c r="V276" t="inlineStr"/>
+      <c r="W276" t="inlineStr"/>
       <c r="X276" t="inlineStr">
         <is>
           <t>no</t>
@@ -32908,16 +32004,8 @@
           <t>https://expomap.ru/expo/transportlight/</t>
         </is>
       </c>
-      <c r="V277" t="inlineStr">
-        <is>
-          <t>https://transport-light.ru/about</t>
-        </is>
-      </c>
-      <c r="W277" t="inlineStr">
-        <is>
-          <t>https://transport-light.ru/about</t>
-        </is>
-      </c>
+      <c r="V277" t="inlineStr"/>
+      <c r="W277" t="inlineStr"/>
       <c r="X277" t="inlineStr">
         <is>
           <t>no</t>
@@ -33028,16 +32116,8 @@
           <t>https://expomap.ru/expo/tsement-beton-suhie-smesi/</t>
         </is>
       </c>
-      <c r="V278" t="inlineStr">
-        <is>
-          <t>https://infocem.info/</t>
-        </is>
-      </c>
-      <c r="W278" t="inlineStr">
-        <is>
-          <t>https://infocem.info/</t>
-        </is>
-      </c>
+      <c r="V278" t="inlineStr"/>
+      <c r="W278" t="inlineStr"/>
       <c r="X278" t="inlineStr">
         <is>
           <t>no</t>
@@ -33141,16 +32221,8 @@
           <t>https://expomap.ru/expo/universe-ecom-convention-globalnaya-cifrovaya-transformaciya-budushego/2026/</t>
         </is>
       </c>
-      <c r="V279" t="inlineStr">
-        <is>
-          <t>https://universeecomconvention.ru</t>
-        </is>
-      </c>
-      <c r="W279" t="inlineStr">
-        <is>
-          <t>https://universeecomconvention.ru</t>
-        </is>
-      </c>
+      <c r="V279" t="inlineStr"/>
+      <c r="W279" t="inlineStr"/>
       <c r="X279" t="inlineStr">
         <is>
           <t>no</t>
@@ -33270,16 +32342,8 @@
           <t>https://expomap.ru/expo/iskusstvo-kukly/</t>
         </is>
       </c>
-      <c r="V280" t="inlineStr">
-        <is>
-          <t>https://xn--b1algbagsvbaljg8i.xn--p1ai/</t>
-        </is>
-      </c>
-      <c r="W280" t="inlineStr">
-        <is>
-          <t>https://xn--b1algbagsvbaljg8i.xn--p1ai/</t>
-        </is>
-      </c>
+      <c r="V280" t="inlineStr"/>
+      <c r="W280" t="inlineStr"/>
       <c r="X280" t="inlineStr">
         <is>
           <t>no</t>
@@ -33498,16 +32562,8 @@
           <t>https://expomap.ru/expo/agrosalon/2026/oct/</t>
         </is>
       </c>
-      <c r="V282" t="inlineStr">
-        <is>
-          <t>https://www.agrosalon.ru/</t>
-        </is>
-      </c>
-      <c r="W282" t="inlineStr">
-        <is>
-          <t>https://www.agrosalon.ru/</t>
-        </is>
-      </c>
+      <c r="V282" t="inlineStr"/>
+      <c r="W282" t="inlineStr"/>
       <c r="X282" t="inlineStr">
         <is>
           <t>no</t>
@@ -34096,16 +33152,8 @@
           <t>https://expomap.ru/expo/russkij-dom-kreativnye-regiony/</t>
         </is>
       </c>
-      <c r="V287" t="inlineStr">
-        <is>
-          <t>https://rdmoscow.ru/?utm_source=tgexpomap</t>
-        </is>
-      </c>
-      <c r="W287" t="inlineStr">
-        <is>
-          <t>https://rdmoscow.ru/?utm_source=tgexpomap</t>
-        </is>
-      </c>
+      <c r="V287" t="inlineStr"/>
+      <c r="W287" t="inlineStr"/>
       <c r="X287" t="inlineStr">
         <is>
           <t>no</t>
@@ -34223,16 +33271,8 @@
           <t>https://expomap.ru/expo/jarmarka-uk/</t>
         </is>
       </c>
-      <c r="V288" t="inlineStr">
-        <is>
-          <t>https://okron.ru/exhibition/2026</t>
-        </is>
-      </c>
-      <c r="W288" t="inlineStr">
-        <is>
-          <t>https://okron.ru/exhibition/2026</t>
-        </is>
-      </c>
+      <c r="V288" t="inlineStr"/>
+      <c r="W288" t="inlineStr"/>
       <c r="X288" t="inlineStr">
         <is>
           <t>no</t>
@@ -34348,16 +33388,8 @@
           <t>https://expomap.ru/expo/edtech-expo/</t>
         </is>
       </c>
-      <c r="V289" t="inlineStr">
-        <is>
-          <t>https://www.edtechexpo.ru/</t>
-        </is>
-      </c>
-      <c r="W289" t="inlineStr">
-        <is>
-          <t>https://www.edtechexpo.ru/</t>
-        </is>
-      </c>
+      <c r="V289" t="inlineStr"/>
+      <c r="W289" t="inlineStr"/>
       <c r="X289" t="inlineStr">
         <is>
           <t>no</t>
@@ -34464,16 +33496,8 @@
           <t>https://expomap.ru/expo/konnaja-rossija/</t>
         </is>
       </c>
-      <c r="V290" t="inlineStr">
-        <is>
-          <t>http://equinerussia.ru/</t>
-        </is>
-      </c>
-      <c r="W290" t="inlineStr">
-        <is>
-          <t>http://equinerussia.ru/</t>
-        </is>
-      </c>
+      <c r="V290" t="inlineStr"/>
+      <c r="W290" t="inlineStr"/>
       <c r="X290" t="inlineStr">
         <is>
           <t>no</t>
@@ -34849,16 +33873,8 @@
           <t>https://expomap.ru/expo/ndt-russia/</t>
         </is>
       </c>
-      <c r="V293" t="inlineStr">
-        <is>
-          <t>https://www.ndt-russia.ru/ru-RU/</t>
-        </is>
-      </c>
-      <c r="W293" t="inlineStr">
-        <is>
-          <t>https://www.ndt-russia.ru/ru-RU/</t>
-        </is>
-      </c>
+      <c r="V293" t="inlineStr"/>
+      <c r="W293" t="inlineStr"/>
       <c r="X293" t="inlineStr">
         <is>
           <t>no</t>
@@ -35179,16 +34195,8 @@
           <t>https://expomap.ru/expo/actuators-engines/</t>
         </is>
       </c>
-      <c r="V296" t="inlineStr">
-        <is>
-          <t>http://www.pcvexpo.ru/en-GB</t>
-        </is>
-      </c>
-      <c r="W296" t="inlineStr">
-        <is>
-          <t>http://www.pcvexpo.ru/en-GB</t>
-        </is>
-      </c>
+      <c r="V296" t="inlineStr"/>
+      <c r="W296" t="inlineStr"/>
       <c r="X296" t="inlineStr">
         <is>
           <t>no</t>
@@ -35421,16 +34429,8 @@
           <t>https://expomap.ru/expo/gassuf/</t>
         </is>
       </c>
-      <c r="V298" t="inlineStr">
-        <is>
-          <t>https://www.gassuf.ru/ru-RU/</t>
-        </is>
-      </c>
-      <c r="W298" t="inlineStr">
-        <is>
-          <t>https://www.gassuf.ru/ru-RU/</t>
-        </is>
-      </c>
+      <c r="V298" t="inlineStr"/>
+      <c r="W298" t="inlineStr"/>
       <c r="X298" t="inlineStr">
         <is>
           <t>no</t>
@@ -35523,16 +34523,8 @@
           <t>https://expomap.ru/expo/aerospace-testing-russia-industrial-testing-control/</t>
         </is>
       </c>
-      <c r="V299" t="inlineStr">
-        <is>
-          <t>http://www.testing-control.ru/en-GB</t>
-        </is>
-      </c>
-      <c r="W299" t="inlineStr">
-        <is>
-          <t>http://www.testing-control.ru/en-GB</t>
-        </is>
-      </c>
+      <c r="V299" t="inlineStr"/>
+      <c r="W299" t="inlineStr"/>
       <c r="X299" t="inlineStr">
         <is>
           <t>no</t>
@@ -35865,16 +34857,8 @@
           <t>https://expomap.ru/expo/diagnopolis/</t>
         </is>
       </c>
-      <c r="V302" t="inlineStr">
-        <is>
-          <t>https://congress.fedlab.ru/exhibition/about/</t>
-        </is>
-      </c>
-      <c r="W302" t="inlineStr">
-        <is>
-          <t>https://congress.fedlab.ru/exhibition/about/</t>
-        </is>
-      </c>
+      <c r="V302" t="inlineStr"/>
+      <c r="W302" t="inlineStr"/>
       <c r="X302" t="inlineStr">
         <is>
           <t>no</t>
@@ -36005,16 +34989,8 @@
           <t>https://expomap.ru/expo/rappa-expo/</t>
         </is>
       </c>
-      <c r="V303" t="inlineStr">
-        <is>
-          <t>https://raapa-expo.ru/</t>
-        </is>
-      </c>
-      <c r="W303" t="inlineStr">
-        <is>
-          <t>https://raapa-expo.ru/</t>
-        </is>
-      </c>
+      <c r="V303" t="inlineStr"/>
+      <c r="W303" t="inlineStr"/>
       <c r="X303" t="inlineStr">
         <is>
           <t>no</t>
@@ -36460,16 +35436,8 @@
           <t>https://expomap.ru/expo/international-exhibition-pir-expo/</t>
         </is>
       </c>
-      <c r="V307" t="inlineStr">
-        <is>
-          <t>http://pirexpo.com/en</t>
-        </is>
-      </c>
-      <c r="W307" t="inlineStr">
-        <is>
-          <t>http://pirexpo.com/en</t>
-        </is>
-      </c>
+      <c r="V307" t="inlineStr"/>
+      <c r="W307" t="inlineStr"/>
       <c r="X307" t="inlineStr">
         <is>
           <t>no</t>
@@ -36587,16 +35555,8 @@
           <t>https://expomap.ru/expo/pir-expo/</t>
         </is>
       </c>
-      <c r="V308" t="inlineStr">
-        <is>
-          <t>https://pirexpo.com/contacts</t>
-        </is>
-      </c>
-      <c r="W308" t="inlineStr">
-        <is>
-          <t>https://pirexpo.com/contacts</t>
-        </is>
-      </c>
+      <c r="V308" t="inlineStr"/>
+      <c r="W308" t="inlineStr"/>
       <c r="X308" t="inlineStr">
         <is>
           <t>no</t>
@@ -36715,16 +35675,8 @@
           <t>https://expomap.ru/expo/reklama/2026/</t>
         </is>
       </c>
-      <c r="V309" t="inlineStr">
-        <is>
-          <t>https://www.reklama-expo.ru/?utm_source=Partners&amp;utm_medium=referral&amp;utm_campaign=expomap.ru_imidz_page</t>
-        </is>
-      </c>
-      <c r="W309" t="inlineStr">
-        <is>
-          <t>https://www.reklama-expo.ru/?utm_source=Partners&amp;utm_medium=referral&amp;utm_campaign=expomap.ru_imidz_page</t>
-        </is>
-      </c>
+      <c r="V309" t="inlineStr"/>
+      <c r="W309" t="inlineStr"/>
       <c r="X309" t="inlineStr">
         <is>
           <t>no</t>
@@ -36958,16 +35910,8 @@
           <t>https://expomap.ru/expo/interlight-smart-city-home-russia/</t>
         </is>
       </c>
-      <c r="V311" t="inlineStr">
-        <is>
-          <t>https://www.interlight-building.ru/</t>
-        </is>
-      </c>
-      <c r="W311" t="inlineStr">
-        <is>
-          <t>https://www.interlight-building.ru/</t>
-        </is>
-      </c>
+      <c r="V311" t="inlineStr"/>
+      <c r="W311" t="inlineStr"/>
       <c r="X311" t="inlineStr">
         <is>
           <t>no</t>
@@ -37081,16 +36025,8 @@
           <t>https://expomap.ru/expo/rimtos/</t>
         </is>
       </c>
-      <c r="V312" t="inlineStr">
-        <is>
-          <t>https://rimtos.ru/</t>
-        </is>
-      </c>
-      <c r="W312" t="inlineStr">
-        <is>
-          <t>https://rimtos.ru/</t>
-        </is>
-      </c>
+      <c r="V312" t="inlineStr"/>
+      <c r="W312" t="inlineStr"/>
       <c r="X312" t="inlineStr">
         <is>
           <t>no</t>
@@ -37213,16 +36149,8 @@
           <t>https://expomap.ru/expo/city-build-russia-moscow/</t>
         </is>
       </c>
-      <c r="V313" t="inlineStr">
-        <is>
-          <t>https://citybuildrussia.tilda.ws/</t>
-        </is>
-      </c>
-      <c r="W313" t="inlineStr">
-        <is>
-          <t>https://citybuildrussia.tilda.ws/</t>
-        </is>
-      </c>
+      <c r="V313" t="inlineStr"/>
+      <c r="W313" t="inlineStr"/>
       <c r="X313" t="inlineStr">
         <is>
           <t>no</t>
@@ -37319,16 +36247,8 @@
           <t>https://expomap.ru/expo/beautiful-houses/</t>
         </is>
       </c>
-      <c r="V314" t="inlineStr">
-        <is>
-          <t>http://www.weg.ru/en</t>
-        </is>
-      </c>
-      <c r="W314" t="inlineStr">
-        <is>
-          <t>http://www.weg.ru/en</t>
-        </is>
-      </c>
+      <c r="V314" t="inlineStr"/>
+      <c r="W314" t="inlineStr"/>
       <c r="X314" t="inlineStr">
         <is>
           <t>no</t>
@@ -38033,16 +36953,8 @@
           <t>https://expomap.ru/expo/global-fresh-market-vegetablesfruits/</t>
         </is>
       </c>
-      <c r="V320" t="inlineStr">
-        <is>
-          <t>https://mosexpo.su/global-fresh-market/</t>
-        </is>
-      </c>
-      <c r="W320" t="inlineStr">
-        <is>
-          <t>https://mosexpo.su/global-fresh-market/</t>
-        </is>
-      </c>
+      <c r="V320" t="inlineStr"/>
+      <c r="W320" t="inlineStr"/>
       <c r="X320" t="inlineStr">
         <is>
           <t>no</t>
@@ -38156,16 +37068,8 @@
           <t>https://expomap.ru/expo/parking-russia/</t>
         </is>
       </c>
-      <c r="V321" t="inlineStr">
-        <is>
-          <t>https://parking-expo.ru/ru-RU/</t>
-        </is>
-      </c>
-      <c r="W321" t="inlineStr">
-        <is>
-          <t>https://parking-expo.ru/ru-RU/</t>
-        </is>
-      </c>
+      <c r="V321" t="inlineStr"/>
+      <c r="W321" t="inlineStr"/>
       <c r="X321" t="inlineStr">
         <is>
           <t>no</t>
@@ -38644,16 +37548,8 @@
           <t>https://expomap.ru/expo/vezdehoder/</t>
         </is>
       </c>
-      <c r="V325" t="inlineStr">
-        <is>
-          <t>https://vezdehoder.ru/</t>
-        </is>
-      </c>
-      <c r="W325" t="inlineStr">
-        <is>
-          <t>https://vezdehoder.ru/</t>
-        </is>
-      </c>
+      <c r="V325" t="inlineStr"/>
+      <c r="W325" t="inlineStr"/>
       <c r="X325" t="inlineStr">
         <is>
           <t>no</t>
@@ -38764,16 +37660,8 @@
           <t>https://expomap.ru/expo/lodki-expo/</t>
         </is>
       </c>
-      <c r="V326" t="inlineStr">
-        <is>
-          <t>https://lodkiexpo.ru/</t>
-        </is>
-      </c>
-      <c r="W326" t="inlineStr">
-        <is>
-          <t>https://lodkiexpo.ru/</t>
-        </is>
-      </c>
+      <c r="V326" t="inlineStr"/>
+      <c r="W326" t="inlineStr"/>
       <c r="X326" t="inlineStr">
         <is>
           <t>no</t>
@@ -38870,16 +37758,8 @@
           <t>https://expomap.ru/expo/moskovskoe-avtoshou/</t>
         </is>
       </c>
-      <c r="V327" t="inlineStr">
-        <is>
-          <t>https://autoshow.moscow</t>
-        </is>
-      </c>
-      <c r="W327" t="inlineStr">
-        <is>
-          <t>https://autoshow.moscow</t>
-        </is>
-      </c>
+      <c r="V327" t="inlineStr"/>
+      <c r="W327" t="inlineStr"/>
       <c r="X327" t="inlineStr">
         <is>
           <t>no</t>
@@ -38997,16 +37877,8 @@
           <t>https://expomap.ru/expo/poehali/</t>
         </is>
       </c>
-      <c r="V328" t="inlineStr">
-        <is>
-          <t>https://poehaliexpo.ru/</t>
-        </is>
-      </c>
-      <c r="W328" t="inlineStr">
-        <is>
-          <t>https://poehaliexpo.ru/</t>
-        </is>
-      </c>
+      <c r="V328" t="inlineStr"/>
+      <c r="W328" t="inlineStr"/>
       <c r="X328" t="inlineStr">
         <is>
           <t>no</t>
@@ -39219,16 +38091,8 @@
           <t>https://expomap.ru/expo/biot/2026/</t>
         </is>
       </c>
-      <c r="V330" t="inlineStr">
-        <is>
-          <t>https://biot-expo.ru/</t>
-        </is>
-      </c>
-      <c r="W330" t="inlineStr">
-        <is>
-          <t>https://biot-expo.ru/</t>
-        </is>
-      </c>
+      <c r="V330" t="inlineStr"/>
+      <c r="W330" t="inlineStr"/>
       <c r="X330" t="inlineStr">
         <is>
           <t>no</t>
@@ -39342,16 +38206,8 @@
           <t>https://expomap.ru/expo/arka/2026/nov/</t>
         </is>
       </c>
-      <c r="V331" t="inlineStr">
-        <is>
-          <t>https://vdnh.ru/arca/</t>
-        </is>
-      </c>
-      <c r="W331" t="inlineStr">
-        <is>
-          <t>https://vdnh.ru/arca/</t>
-        </is>
-      </c>
+      <c r="V331" t="inlineStr"/>
+      <c r="W331" t="inlineStr"/>
       <c r="X331" t="inlineStr">
         <is>
           <t>no</t>
@@ -39460,16 +38316,8 @@
           <t>https://expomap.ru/expo/psycoach-expo/2026/nov/</t>
         </is>
       </c>
-      <c r="V332" t="inlineStr">
-        <is>
-          <t>https://psycoach-expo.ru/</t>
-        </is>
-      </c>
-      <c r="W332" t="inlineStr">
-        <is>
-          <t>https://psycoach-expo.ru/</t>
-        </is>
-      </c>
+      <c r="V332" t="inlineStr"/>
+      <c r="W332" t="inlineStr"/>
       <c r="X332" t="inlineStr">
         <is>
           <t>no</t>
@@ -39949,16 +38797,8 @@
           <t>https://expomap.ru/expo/arsenal/</t>
         </is>
       </c>
-      <c r="V336" t="inlineStr">
-        <is>
-          <t>https://arsenalexpo.ru/?ysclid=mp5rsg8boc755450552</t>
-        </is>
-      </c>
-      <c r="W336" t="inlineStr">
-        <is>
-          <t>https://arsenalexpo.ru/?ysclid=mp5rsg8boc755450552</t>
-        </is>
-      </c>
+      <c r="V336" t="inlineStr"/>
+      <c r="W336" t="inlineStr"/>
       <c r="X336" t="inlineStr">
         <is>
           <t>no</t>
@@ -40074,16 +38914,8 @@
           <t>https://expomap.ru/expo/toolmash/</t>
         </is>
       </c>
-      <c r="V337" t="inlineStr">
-        <is>
-          <t>https://toolmash.ru/</t>
-        </is>
-      </c>
-      <c r="W337" t="inlineStr">
-        <is>
-          <t>https://toolmash.ru/</t>
-        </is>
-      </c>
+      <c r="V337" t="inlineStr"/>
+      <c r="W337" t="inlineStr"/>
       <c r="X337" t="inlineStr">
         <is>
           <t>no</t>
@@ -40198,16 +39030,8 @@
           <t>https://expomap.ru/expo/woodex/</t>
         </is>
       </c>
-      <c r="V338" t="inlineStr">
-        <is>
-          <t>https://woodexpo.ru/ru/</t>
-        </is>
-      </c>
-      <c r="W338" t="inlineStr">
-        <is>
-          <t>https://woodexpo.ru/ru/</t>
-        </is>
-      </c>
+      <c r="V338" t="inlineStr"/>
+      <c r="W338" t="inlineStr"/>
       <c r="X338" t="inlineStr">
         <is>
           <t>no</t>
@@ -40714,16 +39538,8 @@
           <t>https://expomap.ru/expo/promediatech/</t>
         </is>
       </c>
-      <c r="V342" t="inlineStr">
-        <is>
-          <t>https://www.pmtf.ru/pmtf/visiteur/benefits.php?utm_source=expomap</t>
-        </is>
-      </c>
-      <c r="W342" t="inlineStr">
-        <is>
-          <t>https://www.pmtf.ru/pmtf/visiteur/benefits.php?utm_source=expomap</t>
-        </is>
-      </c>
+      <c r="V342" t="inlineStr"/>
+      <c r="W342" t="inlineStr"/>
       <c r="X342" t="inlineStr">
         <is>
           <t>no</t>

</xml_diff>